<commit_message>
used quaterly data to show pie chart
</commit_message>
<xml_diff>
--- a/EXCEL/Column Line , Bar and Pie Chart.xlsx
+++ b/EXCEL/Column Line , Bar and Pie Chart.xlsx
@@ -8,25 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="8_{395BFD57-1E90-4691-ACBA-D83887686582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB2BA4CC-A0A0-4BEC-B138-8B7FFD2177E6}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="8_{395BFD57-1E90-4691-ACBA-D83887686582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BDC812A-5704-4620-A7F3-8678B259ABDC}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{8D6C3E24-154E-4CBF-9FDB-C2144009661E}"/>
+    <workbookView minimized="1" xWindow="1572" yWindow="1440" windowWidth="17280" windowHeight="10500" xr2:uid="{8D6C3E24-154E-4CBF-9FDB-C2144009661E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$A$3:$A$13</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$B$3:$B$13</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$A$3:$A$13</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$B$3:$B$13</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$A$3:$A$13</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$B$3:$B$13</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$A$3:$A$13</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$B$3:$B$13</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Sheet1!$A$3:$A$13</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">Sheet1!$B$3:$B$13</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -48,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Month</t>
   </si>
@@ -94,12 +82,30 @@
   <si>
     <t>Dec</t>
   </si>
+  <si>
+    <t>Quarter report</t>
+  </si>
+  <si>
+    <t>Q1</t>
+  </si>
+  <si>
+    <t>Q2</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Amount/Q</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="16"/>
       <color theme="1"/>
@@ -111,6 +117,12 @@
       <b/>
       <sz val="16"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -136,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -148,6 +160,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1017,6 +1032,272 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$F$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Amount/Q</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$E$2:$E$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Q1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Q2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Q3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Q4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$F$2:$F$5</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>41000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>63000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>81000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>107000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-029F-47B6-A284-CA4F90BF8E44}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1097,6 +1378,43 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="11">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent5"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -2138,20 +2456,539 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>125730</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>253093</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>796290</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>209550</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>670560</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>57149</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2178,16 +3015,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>971550</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>118110</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>2722</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>248739</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>666750</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>194310</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>677635</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>52795</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2207,6 +3044,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>375934</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>8965</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>17929</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0CCBBDC3-6C8B-193A-65F2-D677EA7DC304}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2536,10 +3409,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{883DE418-4CDA-4FE1-82AF-58A22B2F2AC1}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" ht="42" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2549,8 +3422,14 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -2560,8 +3439,15 @@
       <c r="C2" s="3">
         <v>2000</v>
       </c>
+      <c r="E2" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" s="4">
+        <f>SUM(B2:B4)</f>
+        <v>41000</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -2571,8 +3457,15 @@
       <c r="C3" s="3">
         <v>3000</v>
       </c>
+      <c r="E3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="4">
+        <f>SUM(B5:B7)</f>
+        <v>63000</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
@@ -2582,8 +3475,15 @@
       <c r="C4" s="3">
         <v>2500</v>
       </c>
+      <c r="E4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="4">
+        <f>SUM(B8:B10)</f>
+        <v>81000</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
@@ -2593,8 +3493,15 @@
       <c r="C5" s="3">
         <v>4000</v>
       </c>
+      <c r="E5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="4">
+        <f>SUM(B11:B13)</f>
+        <v>107000</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -2605,7 +3512,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>8</v>
       </c>
@@ -2616,7 +3523,7 @@
         <v>7000</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
@@ -2627,7 +3534,7 @@
         <v>6500</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>10</v>
       </c>
@@ -2638,7 +3545,7 @@
         <v>8000</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>11</v>
       </c>
@@ -2649,7 +3556,7 @@
         <v>9000</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
@@ -2660,7 +3567,7 @@
         <v>9500</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A12" s="2" t="s">
         <v>13</v>
       </c>
@@ -2671,7 +3578,7 @@
         <v>10000</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="2" t="s">
         <v>14</v>
       </c>
@@ -2682,10 +3589,11 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="C14" s="4"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
depicted whole data in the form of bar graph
</commit_message>
<xml_diff>
--- a/EXCEL/Column Line , Bar and Pie Chart.xlsx
+++ b/EXCEL/Column Line , Bar and Pie Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="8_{395BFD57-1E90-4691-ACBA-D83887686582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BDC812A-5704-4620-A7F3-8678B259ABDC}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="8_{395BFD57-1E90-4691-ACBA-D83887686582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BED26C0-2CE8-499A-BD3E-BE320C583F65}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1572" yWindow="1440" windowWidth="17280" windowHeight="10500" xr2:uid="{8D6C3E24-154E-4CBF-9FDB-C2144009661E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{8D6C3E24-154E-4CBF-9FDB-C2144009661E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1298,6 +1298,497 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sales</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$13</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>12000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>14000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>18000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>23000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>28000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>30000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>32000</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>35000</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A9D8-4752-B651-C0FDB54945D3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Profit</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$13</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2500</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5500</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6500</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9500</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-A9D8-4752-B651-C0FDB54945D3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="182"/>
+        <c:axId val="480903087"/>
+        <c:axId val="175508271"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="480903087"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="175508271"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="175508271"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="480903087"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1415,6 +1906,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -2633,6 +3164,511 @@
       <cs:styleClr val="auto"/>
     </cs:lnRef>
     <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
@@ -3080,6 +4116,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>363070</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>10885</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>261257</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9626E85A-4028-DDB6-28D2-B8AF98492CD6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3595,6 +4667,7 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
used combo chart to describe the data
</commit_message>
<xml_diff>
--- a/EXCEL/Column Line , Bar and Pie Chart.xlsx
+++ b/EXCEL/Column Line , Bar and Pie Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/898af4500e89e0da/Desktop/DHRUV/Data Science and Analytics with GenAl/EXCEL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="74" documentId="8_{395BFD57-1E90-4691-ACBA-D83887686582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BED26C0-2CE8-499A-BD3E-BE320C583F65}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="8_{395BFD57-1E90-4691-ACBA-D83887686582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D20BBCC-2E41-4B0C-B13D-CF740F0E8E8F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{8D6C3E24-154E-4CBF-9FDB-C2144009661E}"/>
+    <workbookView minimized="1" xWindow="1764" yWindow="1416" windowWidth="17280" windowHeight="10500" xr2:uid="{8D6C3E24-154E-4CBF-9FDB-C2144009661E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1789,6 +1789,576 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Sales</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$2:$B$13</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>12000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>14000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>18000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>20000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>25000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>23000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>28000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>30000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>32000</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>35000</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>40000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-BA20-422C-A5B2-56D68AC8AD71}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="557550031"/>
+        <c:axId val="175493391"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Profit</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>Jan</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Feb</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Mar</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Apr</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>May</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Jun</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Jul</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Aug</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Sep</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Oct</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Nov</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>Dec</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$C$2:$C$13</c:f>
+              <c:numCache>
+                <c:formatCode>#,##0</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2500</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5500</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6500</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9500</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-BA20-422C-A5B2-56D68AC8AD71}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="557569983"/>
+        <c:axId val="175489071"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="557550031"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="175493391"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="175493391"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="557550031"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="175489071"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:numFmt formatCode="#,##0" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="557569983"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="557569983"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="175489071"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1946,6 +2516,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -3979,6 +4589,509 @@
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -4152,6 +5265,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>212271</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>54428</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E1C01E8-A438-7A2C-9A11-DB6B3D162F88}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>